<commit_message>
Added iOS and Android Tests
</commit_message>
<xml_diff>
--- a/src/test/java/mobileAutomation/testData/Testdata.xlsx
+++ b/src/test/java/mobileAutomation/testData/Testdata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bijitbiswas/AutomationProjectTestNG/src/test/java/mobileAutomation/testData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bijitbiswas/AutomationProject-Appium-TestNG/src/test/java/mobileAutomation/testData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03A8DA5E-A597-4A4C-BA2F-C27D05147380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C40555-86F6-DF49-8037-F43C985C7934}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,9 +30,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="4">
   <si>
-    <t>addAndRemoveCartItem</t>
-  </si>
-  <si>
     <t>standard_user</t>
   </si>
   <si>
@@ -40,6 +37,9 @@
   </si>
   <si>
     <t>default_value</t>
+  </si>
+  <si>
+    <t>addItemsToCart</t>
   </si>
 </sst>
 </file>
@@ -404,21 +404,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>